<commit_message>
fix: doc-parser fixes and improvement for llamacpp
+ simplyfied query for doc-parser to improve llama.cpp performance
+ adding env vars for doc-parser
</commit_message>
<xml_diff>
--- a/data/sample_news_with_factoids.xlsx
+++ b/data/sample_news_with_factoids.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>['Chinese researchers identified a new virus', 'The new virus is linked to an illness that has infected dozens of people across Asia', 'The illness has caused fears in a region that was struck by a deadly epidemic on 2003-01-09']</t>
+          <t>['Chinese researchers identified a new virus', 'The new virus is behind an illness', 'The illness has infected dozens of people across Asia', 'The identification of the new virus set off fears in the region', 'The region was struck by a deadly epidemic in 2003']</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>['The spread of a mysterious respiratory virus prompted authorities to limit travel in cities in China on 2020-01-23.', 'The mysterious respiratory virus was first found in Wuhan on 2019-12-01.', 'The mysterious respiratory virus has spread across China.', 'The mysterious respiratory virus has spread to at least 10 other countries.']</t>
+          <t>['The spread of a mysterious respiratory virus prompted the authorities to limit travel in cities in China', 'The authorities are limiting travel in Wuhan', 'The mysterious respiratory virus was first found in Wuhan in December 2019', 'The mysterious respiratory virus spread across China', 'The mysterious respiratory virus spread to at least 10 other countries']</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>['U.S. stock futures are down sharply on 2020-01-27 due to fears about the coronavirus outbreak.']</t>
+          <t>['U.S. stock futures were down sharply on 2020-01-27', 'Fears about the coronavirus outbreak caused U.S. stock futures to be down sharply on 2020-01-27']</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>['As President Trump’s lawyers open the third day of their defense on 2020-01-28, an important question hangs over Washington: Will the Republican-controlled Senate agree to hear testimony from witnesses?', 'When the speaker flew to China at the beginning of January to teach a three-week college class, the Wuhan coronavirus was barely on anyone’s radar.', 'By the time the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world.', 'On 2020-01-24, the Wuhan coronavirus had more than 800 cases in China.', 'By 2020-01-27, the total number of Wuhan coronavirus deaths was at least 80.']</t>
+          <t>["President Trump's lawyers open the third day of their defense on 2020-01-28", 'An important question hangs over Washington regarding whether the Republican-controlled Senate will agree to hear testimony from witnesses', "The Wuhan coronavirus was barely on anyone's radar when the speaker flew to China at the beginning of January to teach a three-week college class", 'When the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world', 'On 2020-01-24, there were more than 800 cases and 26 deaths from the Wuhan coronavirus in China', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80', 'Apple is scheduled to report earnings on 2020-01-28']</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>['The World Health Organization declared a global health emergency on 2020-01-30', 'The coronavirus outbreak spread beyond China on 2020-01-30', 'The coronavirus outbreak emerged in China on 2019-12-01']</t>
+          <t>['The World Health Organization declared a global health emergency on 2020-01-31', 'The coronavirus outbreak spread well beyond China', 'The coronavirus outbreak emerged in China in December 2019']</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>['The observation date is 2020-02-06.', 'The deadly virus nearly paralyzed cities in China and other parts of Asia.', 'Kolmi Hopen is a company located in ANGERS, France.', 'Kolmi Hopen makes medical face masks.', "Medical face masks are currently one of the world's hottest commodities."]</t>
+          <t>['The relentless whir of machines is echoing across a cavernous French factory floor on 2020-02-03', 'The deadly virus nearly paralyzed cities in other parts of Asia', 'Kolmi Hopen makes the medical face mask', 'The medical face mask is suddenly one of the world’s hottest commodities']</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>['Art Basel Hong Kong, an international art market destination, was canceled on 2020-02-07', 'The organizers cited the sudden and widespread outbreak of the coronavirus in China as the reason for the cancellation', 'Art Basel Hong Kong was scheduled to run from March 17 through March 21', 'Japan had several confirmed coronavirus cases when a giant cruise ship arrived at the port of Yokohama on 2020-01-27', 'An alliance between Saudi Arabia and Russia has helped prop up oil prices for the last three years', 'Saudi Arabia and Russia were not in perfect harmony on 2020-02-03 regarding production targets', 'Saudi Arabia and Russia attempted to recalibrate production targets to cope with reduced demand from China', "China's economy has been crippled by the coronavirus epidemic"]</t>
+          <t>['The 2020 edition of Art Basel Hong Kong was canceled', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China for the cancellation of Art Basel Hong Kong', 'Art Basel Hong Kong was held at the Hong Kong Convention and Exhibition Center', 'Art Basel Hong Kong was scheduled to run from March 17 to March 21', 'Japan already had several confirmed coronavirus cases', 'A giant cruise ship arrived at the port of Yokohama on 2020-01-27', 'An alliance between Saudi Arabia and Russia helped prop up oil prices for the last three years', 'Saudi Arabia and Russia tried to recalibrate production targets', 'Saudi Arabia and Russia tried to recalibrate production targets to cope with reduced demand from China', "China's economy was crippled by the coronavirus epidemic"]</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>['On 2020-02-09, the coronavirus epidemic in China surpassed a death toll that exceeds the SARS outbreak death toll from on 2003-02-09', "The development of the coronavirus epidemic's death toll coincided with news that World Health Organization experts might soon be in China to help stanch the crisis"]</t>
+          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09', 'On 2020-02-09, the death toll of the coronavirus epidemic in China exceeded the death toll of the SARS outbreak on 2003-02-09', 'The development regarding the death toll exceeding the SARS outbreak coincided with news that World Health Organization experts might soon be in China', 'World Health Organization experts might soon enter China to help stanch the crisis']</t>
         </is>
       </c>
     </row>
@@ -644,7 +644,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>['As many people across China returned to work on 2020-02-10 after an extended Lunar New Year break', 'China was confronting two bleak statistics on 2020-02-10']</t>
+          <t>['Many people across China returned to work on 2020-02-10', 'The return to work in China occurred after an extended Lunar New Year break', 'China is confronting two bleak statistics']</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>['A family from Shanghai was vacationing in Singapore on 2020-01-01', 'The family learned that the new coronavirus had arrived in Singapore from China', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways when making decisions involving risks', 'The situation described by Tversky and Kahneman is known as the Asian disease problem', 'A woman sick from the coronavirus was released from a San Diego hospital on 2020-02-11', 'The woman was released because a labeling error on samples intended for virus testing led officials to incorrectly indicate that she was not infected', 'Chinese health officials stated on 2020-02-11 that the death toll from the coronavirus had passed 1,000', "Latest updates and maps regarding the virus's reach are available"]</t>
+          <t>['The family from Shanghai was vacationing in Singapore on 2020-01-01.', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China.', 'Humans can be irrational in systematic ways when making decisions that involve risks.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways using a hypothetical situation.', 'The coronavirus epidemic, known as the Asian disease problem, was relevant to the situation demonstrated by Amos Tversky and Daniel Kahneman.', 'Federal authorities said on 2020-02-10 that a woman sick from the coronavirus was released from a San Diego hospital.', 'A labeling error on samples to be tested for the virus led officials to incorrectly indicate that the woman sick from the coronavirus was not infected.', 'Chinese health officials said on 2020-02-11 that the death toll from the coronavirus had passed 1,000.', 'The text provided the latest updates and maps of where the virus had reached.']</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: document parser sequential processing + added HPCpolito installation docs
+ added sequential batches execution on document parser, to respect local server queues
+ edits to env_config
</commit_message>
<xml_diff>
--- a/data/sample_news_with_factoids.xlsx
+++ b/data/sample_news_with_factoids.xlsx
@@ -468,7 +468,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>['Chinese researchers identified a new virus', 'The new virus is behind an illness', 'The illness has infected dozens of people across Asia', 'The identification of the new virus set off fears in the region', 'The region was struck by a deadly epidemic in 2003']</t>
+          <t>['Chinese researchers in Hong Kong identified a new virus', 'The new virus is behind an illness', 'The illness has infected dozens of people across Asia', 'The identification of the new virus set off fears in the region', 'The region was struck by a deadly epidemic on 2003-01-09']</t>
         </is>
       </c>
     </row>
@@ -490,7 +490,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>['The spread of a mysterious respiratory virus prompted the authorities to limit travel in cities in China', 'The authorities are limiting travel in Wuhan', 'The mysterious respiratory virus was first found in Wuhan in December 2019', 'The mysterious respiratory virus spread across China', 'The mysterious respiratory virus spread to at least 10 other countries']</t>
+          <t>['The spread of a mysterious respiratory virus prompted the authorities to limit travel in cities in China', 'The cities in China affected by travel limits include Wuhan', 'The mysterious respiratory virus was first found in Wuhan in December 2019', 'The mysterious respiratory virus spread across China', 'The mysterious respiratory virus spread to at least 10 other countries']</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>['U.S. stock futures were down sharply on 2020-01-27', 'Fears about the coronavirus outbreak caused U.S. stock futures to be down sharply on 2020-01-27']</t>
+          <t>['U.S. stock futures were down sharply on 2020-01-27', 'The decline of U.S. stock futures on 2020-01-27 was due to fears about the coronavirus outbreak']</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>["President Trump's lawyers open the third day of their defense on 2020-01-28", 'An important question hangs over Washington regarding whether the Republican-controlled Senate will agree to hear testimony from witnesses', "The Wuhan coronavirus was barely on anyone's radar when the speaker flew to China at the beginning of January to teach a three-week college class", 'When the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world', 'On 2020-01-24, there were more than 800 cases and 26 deaths from the Wuhan coronavirus in China', 'By 2020-01-27, the total number of deaths from the Wuhan coronavirus was at least 80', 'Apple is scheduled to report earnings on 2020-01-28']</t>
+          <t>["President Trump's lawyers open the third day of their defense on 2020-01-28", 'An important question hangs over Washington regarding whether the Republican-controlled Senate will agree to hear testimony from witnesses', 'When the speaker flew to China at the beginning of January to teach a three-week college class, the Wuhan coronavirus was barely on anyone’s radar', 'When the speaker got back to New York on 2020-01-24, the Wuhan coronavirus was front page news around the world', 'On 2020-01-24, the Wuhan coronavirus had more than 800 cases in China', 'By 2020-01-27, the total number of Wuhan coronavirus deaths was at least 80', 'Apple is scheduled to report earnings on 2020-01-28']</t>
         </is>
       </c>
     </row>
@@ -556,7 +556,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>['The World Health Organization declared a global health emergency on 2020-01-31', 'The coronavirus outbreak spread well beyond China', 'The coronavirus outbreak emerged in China in December 2019']</t>
+          <t>['The World Health Organization declared a global health emergency on 2020-01-30', 'The coronavirus outbreak spread well beyond China', 'The coronavirus outbreak emerged in China on 2019-12-01']</t>
         </is>
       </c>
     </row>
@@ -578,7 +578,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>['The relentless whir of machines is echoing across a cavernous French factory floor on 2020-02-03', 'The deadly virus nearly paralyzed cities in other parts of Asia', 'Kolmi Hopen makes the medical face mask', 'The medical face mask is suddenly one of the world’s hottest commodities']</t>
+          <t>['The whir of machines is echoing across a French factory floor around 2020-02-06', 'The echoing of machines in the French factory is an unexpected result of the deadly virus', 'The deadly virus nearly paralyzed cities in other parts of Asia', 'Kolmi Hopen is the company mentioned in the text', 'Kolmi Hopen makes the medical face mask', "The medical face mask is one of the world's hottest commodities"]</t>
         </is>
       </c>
     </row>
@@ -600,7 +600,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>['The 2020 edition of Art Basel Hong Kong was canceled', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China for the cancellation of Art Basel Hong Kong', 'Art Basel Hong Kong was held at the Hong Kong Convention and Exhibition Center', 'Art Basel Hong Kong was scheduled to run from March 17 to March 21', 'Japan already had several confirmed coronavirus cases', 'A giant cruise ship arrived at the port of Yokohama on 2020-01-27', 'An alliance between Saudi Arabia and Russia helped prop up oil prices for the last three years', 'Saudi Arabia and Russia tried to recalibrate production targets', 'Saudi Arabia and Russia tried to recalibrate production targets to cope with reduced demand from China', "China's economy was crippled by the coronavirus epidemic"]</t>
+          <t>['The edition of Art Basel Hong Kong for 2020 was canceled', 'Organizers cited the sudden and widespread outbreak of the coronavirus in China for the cancellation of Art Basel Hong Kong', 'The fair, Art Basel Hong Kong, was held at the Hong Kong Convention and Exhibition Center', 'Art Basel Hong Kong was scheduled to run from March 17 through March 21', 'Japan already had several confirmed coronavirus cases', 'A giant cruise ship arrived at the port of Yokohama on 2020-01-27', 'An alliance between Saudi Arabia and Russia helped prop up oil prices for the last three years', 'Saudi Arabia and Russia were not in perfect harmony on 2020-02-03', 'Saudi Arabia and Russia tried to recalibrate production targets to cope with reduced demand from China', "China's economy was crippled by the coronavirus epidemic"]</t>
         </is>
       </c>
     </row>
@@ -622,7 +622,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09', 'On 2020-02-09, the death toll of the coronavirus epidemic in China exceeded the death toll of the SARS outbreak on 2003-02-09', 'The development regarding the death toll exceeding the SARS outbreak coincided with news that World Health Organization experts might soon be in China', 'World Health Organization experts might soon enter China to help stanch the crisis']</t>
+          <t>['The coronavirus epidemic in China surpassed a grim milestone on 2020-02-09', 'The death toll of the coronavirus epidemic in China on 2020-02-09 exceeded the death toll of the SARS outbreak on 2003-02-09', 'The development regarding the coronavirus epidemic in China coincided with news that World Health Organization experts might soon be in China', 'World Health Organization experts might soon enter China to help stanch the coronavirus crisis']</t>
         </is>
       </c>
     </row>
@@ -666,7 +666,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>['The family from Shanghai was vacationing in Singapore on 2020-01-01.', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China.', 'Humans can be irrational in systematic ways when making decisions that involve risks.', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways using a hypothetical situation.', 'The coronavirus epidemic, known as the Asian disease problem, was relevant to the situation demonstrated by Amos Tversky and Daniel Kahneman.', 'Federal authorities said on 2020-02-10 that a woman sick from the coronavirus was released from a San Diego hospital.', 'A labeling error on samples to be tested for the virus led officials to incorrectly indicate that the woman sick from the coronavirus was not infected.', 'Chinese health officials said on 2020-02-11 that the death toll from the coronavirus had passed 1,000.', 'The text provided the latest updates and maps of where the virus had reached.']</t>
+          <t>['The family from Shanghai was vacationing in Singapore on 2020-01-01', 'The family from Shanghai learned that the new coronavirus arrived in Singapore from China while the family from Shanghai was vacationing in Singapore on 2020-01-01', 'Humans can be irrational in systematic ways when making decisions that involve risks', 'Psychologists Amos Tversky and Daniel Kahneman demonstrated that humans can be irrational in systematic ways using a hypothetical situation', 'The coronavirus epidemic, known as the Asian disease problem, was relevant to the demonstration by Amos Tversky and Daniel Kahneman', 'Federal authorities said on 2020-02-10 that a woman sick from the coronavirus was released from a San Diego hospital', 'The release of the woman sick from the coronavirus occurred after a labeling error on samples to be tested for the virus', 'The labeling error on samples led officials to incorrectly indicate that the woman sick from the coronavirus was not infected', 'Chinese health officials said on 2020-02-11 that the death toll from the coronavirus had passed 1,000', 'The text provided the latest updates and maps of where the virus has reached']</t>
         </is>
       </c>
     </row>

</xml_diff>